<commit_message>
feat: terminologia FMR en espanol (Vaquero Completo, Lazo por Parejas)
Alinea etiquetas publicas con el Reglamento FMR: Vaquero Completo, cabecero/pialador, categoria Master; confirma dinero 50/50 y deja IDs internos estables.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/evento-manual.xlsx
+++ b/templates/evento-manual.xlsx
@@ -7,13 +7,13 @@
     <sheet sheetId="1" name="Cómo llenar" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Evento" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Barriles" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Barriles Masters" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="Barriles Master" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Lazo de Becerro" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Lazo en Falso" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Achatada de Novillos" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Amarre de Chiva" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Team Roping" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Team Roping Masters" state="visible" r:id="rId13"/>
+    <sheet sheetId="9" name="Lazo por Parejas" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Lazo por Parejas Master" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="Caballo con Pretal" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="Caballo con Montura" state="visible" r:id="rId15"/>
     <sheet sheetId="13" name="Jineteos de Toros" state="visible" r:id="rId16"/>
@@ -26,7 +26,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="84">
   <si>
-    <t>ArenaPro Stats · Plantilla manual FMR Tour</t>
+    <t>ArenaPro Estadísticas · Plantilla manual FMR Tour</t>
   </si>
   <si>
     <t>¿Para qué sirve?</t>
@@ -56,7 +56,7 @@
     <t>4. Columnas según disciplina</t>
   </si>
   <si>
-    <t>Tiempos: Ronda 1–3 + Total. Jineteos/Montura/Pretal: solo Calificación. Team Roping: Cabecero + Pialador (sin Rol).</t>
+    <t>Tiempos: Ronda 1–3 + Total. Jineteos/Montura/Pretal: solo Calificación. Lazo por Parejas: Cabecero + Pialador (sin Rol).</t>
   </si>
   <si>
     <t>5. NT / NP en tiempos</t>
@@ -65,16 +65,16 @@
     <t>En rondas: NT, NP, o 60 (= NT). En Achatada: 120 (= NT).</t>
   </si>
   <si>
-    <t>6. Team Roping</t>
+    <t>6. Lazo por Parejas</t>
   </si>
   <si>
-    <t>Solo 2 hojas (Abierta y Masters). Una fila = Cabecero + Pialador (columnas distintas). Ronda 1 está en la columna H (no en G: ahí va el dinero). Stats parte cada dúo a Headers y Heelers.</t>
+    <t>Solo 2 hojas (Abierta y Master). Una fila = Cabecero + Pialador (columnas distintas). Ronda 1 está en la columna H (no en G: ahí va el dinero). Estadísticas parte cada dúo a Cabeceros y Pialadores (dinero 50/50).</t>
   </si>
   <si>
     <t>7. Publicar</t>
   </si>
   <si>
-    <t>Guarda el .xlsx → publicar.bat → admin → suelta el archivo → preview → Agregar a Stats → Publicar.</t>
+    <t>Guarda el .xlsx → publicar.bat → admin → suelta el archivo → preview → Agregar a Estadísticas → Publicar.</t>
   </si>
   <si>
     <t>Datos del evento (obligatorio)</t>
@@ -173,10 +173,10 @@
     <t>En rondas: NT, NP o 60 (=NT). Dinero sin decimales. Sin lugar = no clasificó.</t>
   </si>
   <si>
-    <t>Clasificación final · Barriles Masters</t>
+    <t>Clasificación final · Barriles Master</t>
   </si>
   <si>
-    <t>Barriles Masters</t>
+    <t>Barriles Master</t>
   </si>
   <si>
     <t>Clasificación final · Lazo de Becerro</t>
@@ -209,13 +209,13 @@
     <t>Amarre de Chiva</t>
   </si>
   <si>
-    <t>Clasificación final · Team Roping</t>
+    <t>Clasificación final · Lazo por Parejas</t>
   </si>
   <si>
-    <t>Lugar = puesto final. Cabecero + Pialador por fila (Stats parte Header/Heeler). Rondas: NT/NP o 60=NT. Sin lugar = no clasificó.</t>
+    <t>Lugar = puesto final. Cabecero + Pialador por fila (parte Cabecero/Pialador). Rondas: NT/NP o 60=NT. Sin lugar = no clasificó.</t>
   </si>
   <si>
-    <t>Team Roping</t>
+    <t>Lazo por Parejas</t>
   </si>
   <si>
     <t>Cabecero</t>
@@ -233,10 +233,10 @@
     <t>Cabecero + Pialador por fila. En rondas: NT, NP o 60 (=NT). Sin lugar = no clasificó.</t>
   </si>
   <si>
-    <t>Clasificación final · Team Roping Masters</t>
+    <t>Clasificación final · Lazo por Parejas Master</t>
   </si>
   <si>
-    <t>Team Roping Masters</t>
+    <t>Lazo por Parejas Master</t>
   </si>
   <si>
     <t>Clasificación final · Caballo con Pretal</t>

</xml_diff>

<commit_message>
Auditoría prelanzamiento: integridad de datos, seguridad del admin, deploy con tests, nombres en MAYÚSCULAS
- Quita evento Truckmania manual duplicado; detector de rodeos duplicados en ingest y al publicar.
- AERCH Circuito 2027 como circuito principal; publicar bloquea principal vacío.
- Consola local: valida Host/Origin + token por sesión (CSRF / DNS rebinding).
- Colisión de id/archivo de evento ya no sobrescribe otro rodeo.
- Publicar corre tests; deploy de Pages por Actions solo con archivos del sitio.
- Aliases por asociación.
- Nombres siempre en MAYÚSCULAS (Excel, ingest, rebuild, sitio).
- Contraste AA, metodología en lenguaje de rodeo, OG/404/robots, noindex admin, cache busting.
- Contraseña de portal 14+, sesión expira a 30 días, override uuid (0 vulnerabilidades).
- ESLint en CI; tests de servidor y de datos publicados.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/evento-manual.xlsx
+++ b/templates/evento-manual.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="86">
   <si>
     <t>ArenaPro Estadísticas · Plantilla manual de evento</t>
   </si>
@@ -71,7 +71,13 @@
     <t>Solo 2 hojas (Abierta y Master). Una fila = Cabecero + Pialador (columnas distintas). Ronda 1 está en la columna H (no en G: ahí va el dinero). Estadísticas parte cada dúo a Cabeceros y Pialadores (dinero 50/50).</t>
   </si>
   <si>
-    <t>7. Publicar</t>
+    <t>7. Nombres en MAYÚSCULAS</t>
+  </si>
+  <si>
+    <t>Escribe los nombres como quieras (mayúsculas, minúsculas o mezcla): al publicar, Estadísticas los convierte a MAYÚSCULAS (juan pérez → JUAN PÉREZ) para que todos los resultados se vean iguales.</t>
+  </si>
+  <si>
+    <t>8. Publicar</t>
   </si>
   <si>
     <t>Guarda el .xlsx → publicar.bat → admin → suelta el archivo → preview → Agregar a Estadísticas → Publicar.</t>
@@ -164,7 +170,7 @@
     <t>Notas</t>
   </si>
   <si>
-    <t>Ejemplo Competidor</t>
+    <t>EJEMPLO COMPETIDOR</t>
   </si>
   <si>
     <t>Borra esta fila; es solo guía</t>
@@ -224,10 +230,10 @@
     <t>Pialador</t>
   </si>
   <si>
-    <t>Ejemplo Cabecero</t>
+    <t>EJEMPLO CABECERO</t>
   </si>
   <si>
-    <t>Ejemplo Pialador</t>
+    <t>EJEMPLO PIALADOR</t>
   </si>
   <si>
     <t>Cabecero + Pialador por fila. En rondas: NT, NP o 60 (=NT). Sin lugar = no clasificó.</t>
@@ -763,7 +769,7 @@
   <sheetPr>
     <tabColor rgb="FFDD9219"/>
   </sheetPr>
-  <dimension ref="B1:C11"/>
+  <dimension ref="B1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -839,6 +845,14 @@
       </c>
       <c r="C11" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -870,7 +884,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -885,7 +899,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -900,59 +914,59 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -960,10 +974,10 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10">
@@ -983,7 +997,7 @@
         <f>IF(COUNTA(H7:J7)=0,"",SUM(H7:J7))</f>
       </c>
       <c r="L7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -1573,7 +1587,7 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -1592,6 +1606,14 @@
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="B48:L48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:D46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:D46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1617,7 +1639,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1628,7 +1650,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -1639,47 +1661,47 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -1687,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -1700,7 +1722,7 @@
         <v>85</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -2056,7 +2078,7 @@
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -2071,6 +2093,14 @@
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B48:H48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2096,7 +2126,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2107,7 +2137,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -2118,47 +2148,47 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -2166,7 +2196,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -2179,7 +2209,7 @@
         <v>85</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -2535,7 +2565,7 @@
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -2550,6 +2580,14 @@
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B48:H48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2575,7 +2613,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2586,7 +2624,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -2597,47 +2635,47 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -2645,7 +2683,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -2658,7 +2696,7 @@
         <v>85</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -3014,7 +3052,7 @@
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -3029,6 +3067,14 @@
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B48:H48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3054,7 +3100,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3068,7 +3114,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -3082,56 +3128,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -3139,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -3157,7 +3203,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -3708,7 +3754,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -3726,6 +3772,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3747,58 +3801,58 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="D4" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -3833,7 +3887,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3847,7 +3901,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -3861,56 +3915,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -3918,7 +3972,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -3938,7 +3992,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -4489,7 +4543,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -4507,6 +4561,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -4532,7 +4594,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -4546,7 +4608,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -4560,56 +4622,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -4617,7 +4679,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -4637,7 +4699,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -5188,7 +5250,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -5206,6 +5268,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5231,7 +5301,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -5245,7 +5315,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -5259,56 +5329,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -5316,7 +5386,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -5336,7 +5406,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -5887,7 +5957,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -5905,6 +5975,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -5930,7 +6008,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -5944,7 +6022,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -5958,56 +6036,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -6015,7 +6093,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -6035,7 +6113,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -6586,7 +6664,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -6604,6 +6682,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6629,7 +6715,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -6643,7 +6729,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -6657,56 +6743,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -6714,7 +6800,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -6734,7 +6820,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -7285,7 +7371,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -7303,6 +7389,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -7328,7 +7422,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -7342,7 +7436,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -7356,56 +7450,56 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -7413,7 +7507,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10">
@@ -7433,7 +7527,7 @@
         <f>IF(COUNTA(G7:I7)=0,"",SUM(G7:I7))</f>
       </c>
       <c r="K7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -7984,7 +8078,7 @@
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -8002,6 +8096,14 @@
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B48:K48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -8027,7 +8129,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -8042,7 +8144,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -8057,59 +8159,59 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -8117,10 +8219,10 @@
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10">
@@ -8140,7 +8242,7 @@
         <f>IF(COUNTA(H7:J7)=0,"",SUM(H7:J7))</f>
       </c>
       <c r="L7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -8730,7 +8832,7 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -8749,6 +8851,14 @@
     <mergeCell ref="B2:L2"/>
     <mergeCell ref="B48:L48"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:D46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:D46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Ronda 2 de auditoría: sync seguro, legales, monitor, E2E, fuente local y CSP
- Publicar: la sincronización solo resuelve sola conflictos en data/circuitos; cualquier otro aborta sin perder el commit local.
- Deploy también tras el workflow Rebuild temporada; E2E con Playwright antes de desplegar.
- Aviso de privacidad, términos y 'Reportar un error' (soporte@arenapro.mx).
- Notas de jueces y aliases fuera del sitio público; en Excel las notas ya no se ven en el detalle.
- Monitor cada hora (disponibilidad, datos, archivos internos, versión vs main) con issue automático.
- Fuente Archivo alojada en el sitio, Content-Security-Policy, sitemap y JSON-LD.
- Errores de carga con mensaje amigable.
- Runbook de operación.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/evento-manual.xlsx
+++ b/templates/evento-manual.xlsx
@@ -167,7 +167,7 @@
     <t>Total tiempos</t>
   </si>
   <si>
-    <t>Notas</t>
+    <t>Notas internas (no se publican)</t>
   </si>
   <si>
     <t>EJEMPLO COMPETIDOR</t>
@@ -879,7 +879,7 @@
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
@@ -1634,7 +1634,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -2121,7 +2121,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -2608,7 +2608,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -3095,7 +3095,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -3882,7 +3882,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -4589,7 +4589,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -5296,7 +5296,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -6003,7 +6003,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -6710,7 +6710,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -7417,7 +7417,7 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
@@ -8124,7 +8124,7 @@
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: marcas en la ficha, Cowboy Protection, CSV del portal y ligas cortas por asociación
- Ficha del competidor: victorias, podios, mejor lugar y por disciplina mejor recorrido, mejor rodeo y promedio (web/lib/marcas.mjs; el rebuild las guarda en historial).

- Cowboy Protection como disciplina propia, calificada por jueces; se reconoce por nombre aunque Time la mande como Jineteos. Nueva hoja en la plantilla de Excel.

- Portal: descarga de tablas en CSV para Excel (clasificación con puntos por rodeo y Vaquero Completo).

- Ligas cortas estadisticas.arenapro.mx/{asociacionId} que redirigen al portal (build y servidor local).

- publicar.bat avisa si falta Node.js.
</commit_message>
<xml_diff>
--- a/templates/evento-manual.xlsx
+++ b/templates/evento-manual.xlsx
@@ -17,14 +17,15 @@
     <sheet sheetId="11" name="Caballo con Pretal" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="Caballo con Montura" state="visible" r:id="rId15"/>
     <sheet sheetId="13" name="Jineteos de Toros" state="visible" r:id="rId16"/>
-    <sheet sheetId="14" name="Polos" state="visible" r:id="rId17"/>
+    <sheet sheetId="14" name="Cowboy Protection" state="visible" r:id="rId17"/>
+    <sheet sheetId="15" name="Polos" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="88">
   <si>
     <t>ArenaPro Estadísticas · Plantilla manual de evento</t>
   </si>
@@ -56,7 +57,7 @@
     <t>4. Columnas según disciplina</t>
   </si>
   <si>
-    <t>Tiempos: Ronda 1–3 + Total. Jineteos/Montura/Pretal: solo Calificación. Lazo por Parejas: Cabecero + Pialador (sin Rol).</t>
+    <t>Tiempos: Ronda 1–3 + Total. Jineteos/Cowboy Protection/Montura/Pretal: solo Calificación. Lazo por Parejas: Cabecero + Pialador (sin Rol).</t>
   </si>
   <si>
     <t>5. NT / NP en tiempos</t>
@@ -276,6 +277,12 @@
   </si>
   <si>
     <t>Jineteos de Toros</t>
+  </si>
+  <si>
+    <t>Clasificación final · Cowboy Protection</t>
+  </si>
+  <si>
+    <t>Cowboy Protection</t>
   </si>
   <si>
     <t>Clasificación final · Polos</t>
@@ -3085,6 +3092,493 @@
   <sheetPr>
     <tabColor rgb="FFDD9219"/>
   </sheetPr>
+  <dimension ref="B1:H48"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="10">
+        <v>1</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10">
+        <v>100</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <v>85</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="12"/>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="12"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="12"/>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="12"/>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+      <c r="H45" s="12"/>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="12"/>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B48" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B48:H48"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C10:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Nombre del competidor" prompt="Escríbelo como quieras: al publicar se convierte a MAYÚSCULAS (ej. juan pérez → JUAN PÉREZ)." sqref="C7:C46">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FFDD9219"/>
+  </sheetPr>
   <dimension ref="B1:K48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -3100,7 +3594,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3131,7 +3625,7 @@
         <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>35</v>

</xml_diff>